<commit_message>
chore(assets): regenerate canonical Item Master Standard v2.2 with GST slab governance
- v2.2.xlsx: clean regeneration via remediate_item_master_standard.py (file unlocked)
  GST_RATE_PERCENT added to Validation Lists col 20 (T): values [0, 5, 12, 18]
  DataValidation BLOCK rule on AA5:AA500 in Item Master Template
  IM-013 appended to Validation Rules sheet
  All v2.2 formula upgrades applied (AI/AJ validation formulas, SKU_PREVIEW)
  File size 33KB -> 144KB (was a stub; now fully populated)

- v2.1.xlsx: in-place formula remediation applied (soft DataValidation alerts)

- Temp file SMRITI_Item_Master_Creation_Standard_v2.2_gst.xlsx removed

Workbook seeder now reads GST_RATE_PERCENT directly from col T:
  'gst_rate: added 0 new values, 4 total active' (idempotent re-run confirmed)

Alembic commands documented in .env comments (gitignored, local dev only)
</commit_message>
<xml_diff>
--- a/assets/Itemmasters/SMRITI_Item_Master_Creation_Standard_v2.1.xlsx
+++ b/assets/Itemmasters/SMRITI_Item_Master_Creation_Standard_v2.1.xlsx
@@ -34,6 +34,7 @@
     <definedName name="List_VENDOR_CODE">'Validation Lists'!$N$2:$N$100</definedName>
     <definedName name="List_WAREHOUSE_CODE">'Validation Lists'!$S$2:$S$20</definedName>
     <definedName name="List_YN">'Validation Lists'!$Q$2:$Q$3</definedName>
+    <definedName name="List_GST_RATE_PERCENT">'Validation Lists'!$T$2:$T$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Creation Workflow'!$A$4:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Item Master Template'!$A$4:$AI$500</definedName>
   </definedNames>
@@ -26509,7 +26510,7 @@
       <formula>AND(J5&lt;&gt;"",I5&lt;&gt;"",J5&gt;I5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="21">
+  <dataValidations count="22">
     <dataValidation sqref="C5:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Dimension Notice" error="Value is not in standard list. SMRITI will validate or onboard this master dimension during import." type="list" errorStyle="warning">
       <formula1>List_ARTICLE_STYLE_CODE</formula1>
     </dataValidation>
@@ -26574,6 +26575,9 @@
     <dataValidation sqref="AH5:AH500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Dimension Notice" error="Value is not in standard list. SMRITI will validate or onboard this master dimension during import." type="list" errorStyle="warning">
       <formula1>List_CREATION_STATUS</formula1>
     </dataValidation>
+    <dataValidation sqref="AA5:AA500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid GST Rate" error="Only statutory GST slabs are permitted: 0%, 5%, 12%, or 18%." promptTitle="GST Rate (%)" prompt="Select 0, 5, 12 or 18" type="list" errorStyle="stop">
+      <formula1>'Validation Lists'!$T$2:$T$6</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -26961,7 +26965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="42" customWidth="1" style="21" min="1" max="1"/>
@@ -27433,6 +27437,138 @@
         </is>
       </c>
       <c r="D23" t="inlineStr">
+        <is>
+          <t>Produces clean preview strings during drafting</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Empty rows displayed permanent ERROR status due to COUNTA evaluating formula empty strings</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Col AI</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Updated formula to IF(AND(A5="",C5=""),"EMPTY",...)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Eliminates 492 false ERROR cells on blank rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COUNTIF on empty SKU_PREVIEW caused false Duplicate SKU_PREVIEW error on blank rows</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Col AJ</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Guarded COUNTIF with AND(B5&lt;&gt;"", COUNTIF(...)&gt;1)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Eliminates 492 false positive duplicate alarms on new row entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Contradiction where missing mandatory attributes showed ERROR in Col AI but OK in Col AJ</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Col AJ</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Added Missing Mandatory Attributes branch in formula</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Synchronizes Col AI status with Col AJ message</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Validation Lists defined ranges were hardcoded to 1-2 cells, blocking standard colors/sizes/brands</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Validation Lists</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Expanded defined ranges (10 to 100 items) with comprehensive retail catalog values</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Allows multi-brand, multi-category retail entry without Excel range lockouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GST 2.0 dynamic threshold had no explicit validation rule</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Validation Rules</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Added Rule IM-013 flagging Selling Price &gt; Rs. 2,500 with GST &lt;= 5%</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Guarantees statutory tax compliance visibility before import</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SKU_PREVIEW formula generated double/trailing hyphens when attributes were empty</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Col B</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Updated formula with conditional delimiters</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>Produces clean preview strings during drafting</t>
         </is>
@@ -28482,7 +28618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S119"/>
+  <dimension ref="A1:T119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28581,6 +28717,11 @@
           <t>WAREHOUSE_CODE</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>GST_RATE_PERCENT</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -28678,6 +28819,11 @@
           <t>WH-MAIN</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -28775,6 +28921,11 @@
           <t>WH-STORE-01</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -28867,6 +29018,11 @@
           <t>CENTRAL-WH</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -28957,6 +29113,11 @@
       <c r="S5" t="inlineStr">
         <is>
           <t>RETAIL-STORE</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>

</xml_diff>